<commit_message>
Commit all changes on Work PC between 1404/10/18 at 1404/11/05 at 11:44
</commit_message>
<xml_diff>
--- a/Distributed systems.xlsx
+++ b/Distributed systems.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project(s)\Python\MyPython2\Python-2024\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\B.Pourtavakoli\Project(s)\Python\My Python Source(s) 14031130\MyPython2\Python-2024\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B1A85DB-6641-4DCC-BE74-80F045B8BF44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{CB93F9FC-27FD-46EE-8180-32B8C0589FD8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -57,7 +56,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0_ ;[Red]\-#,##0\ "/>
   </numFmts>
@@ -624,7 +623,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{745F7B22-BAB1-4AE2-A0CB-3EFE07828C6D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I11"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.45"/>
   <cols>
@@ -843,7 +842,7 @@
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>
       <c r="I8" s="10">
-        <f t="shared" ref="I7:I8" si="1">SUM(B8:H8)</f>
+        <f t="shared" ref="I8" si="1">SUM(B8:H8)</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>